<commit_message>
Fixed bugs on file export to excel and added comments
</commit_message>
<xml_diff>
--- a/loan.xlsx
+++ b/loan.xlsx
@@ -8,13 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="active" sheetId="1" r:id="rId1"/>
+    <sheet name="finished" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="11">
   <si>
     <t>name</t>
   </si>
@@ -40,13 +41,13 @@
     <t>total_payment</t>
   </si>
   <si>
-    <t>ncol</t>
-  </si>
-  <si>
-    <t>wew</t>
-  </si>
-  <si>
-    <t>qwe</t>
+    <t>aa</t>
+  </si>
+  <si>
+    <t>balance</t>
+  </si>
+  <si>
+    <t>nn</t>
   </si>
 </sst>
 </file>
@@ -382,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -416,16 +417,81 @@
         <v>8</v>
       </c>
       <c r="B2">
+        <v>25000</v>
+      </c>
+      <c r="C2">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1">
+        <v>46114</v>
+      </c>
+      <c r="E2" s="1">
+        <v>46236</v>
+      </c>
+      <c r="F2">
+        <v>30000</v>
+      </c>
+      <c r="G2">
+        <v>7500</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2">
         <v>20000</v>
       </c>
       <c r="C2">
         <v>5</v>
       </c>
       <c r="D2" s="1">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="E2" s="1">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="F2">
         <v>25000</v>
@@ -434,58 +500,9 @@
         <v>5000</v>
       </c>
       <c r="H2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3">
-        <v>10000</v>
-      </c>
-      <c r="C3">
-        <v>5</v>
-      </c>
-      <c r="D3" s="1">
-        <v>46112</v>
-      </c>
-      <c r="E3" s="1">
-        <v>46265</v>
-      </c>
-      <c r="F3">
-        <v>12500</v>
-      </c>
-      <c r="G3">
-        <v>2500</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4">
-        <v>15000</v>
-      </c>
-      <c r="C4">
-        <v>6</v>
-      </c>
-      <c r="D4" s="1">
-        <v>46112</v>
-      </c>
-      <c r="E4" s="1">
-        <v>46295</v>
-      </c>
-      <c r="F4">
-        <v>19500</v>
-      </c>
-      <c r="G4">
-        <v>3250</v>
-      </c>
-      <c r="H4">
+        <v>25000</v>
+      </c>
+      <c r="I2">
         <v>0</v>
       </c>
     </row>

</xml_diff>